<commit_message>
#63 complete the draw of the 30 pending repositories in the gold-standard sheets
</commit_message>
<xml_diff>
--- a/lab03/dados/amostra_ouro/amostra_ouro_gabriel.xlsx
+++ b/lab03/dados/amostra_ouro/amostra_ouro_gabriel.xlsx
@@ -1492,13 +1492,17 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr"/>
+          <t>1.91.0</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-30T18:29:40+00:00</t>
+        </is>
+      </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/rust-lang/rust/releases</t>
+          <t>https://github.com/rust-lang/rust/releases/tag/1.91.0</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
@@ -1525,13 +1529,17 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr"/>
+          <t>1.92.0</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-11T14:58:25+00:00</t>
+        </is>
+      </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/rust-lang/rust/releases</t>
+          <t>https://github.com/rust-lang/rust/releases/tag/1.92.0</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
@@ -1558,13 +1566,17 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr"/>
+          <t>1.96.0</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-28T17:50:42+00:00</t>
+        </is>
+      </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/rust-lang/rust/releases</t>
+          <t>https://github.com/rust-lang/rust/releases/tag/1.96.0</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -1591,13 +1603,17 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr"/>
+          <t>1.97.0</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09T12:25:16+00:00</t>
+        </is>
+      </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/rust-lang/rust/releases</t>
+          <t>https://github.com/rust-lang/rust/releases/tag/1.97.0</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
@@ -1624,13 +1640,17 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr"/>
+          <t>1.98.0</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-20T18:05:33+00:00</t>
+        </is>
+      </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/rust-lang/rust/releases</t>
+          <t>https://github.com/rust-lang/rust/releases/tag/1.98.0</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -1842,13 +1862,17 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr"/>
+          <t>agent-skills-v0.699.0</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:28:41+00:00</t>
+        </is>
+      </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/PostHog/posthog/releases</t>
+          <t>https://github.com/PostHog/posthog/releases/tag/agent-skills-v0.699.0</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
@@ -1875,13 +1899,17 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr"/>
+          <t>desktop-v0.61.126</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-31T01:34:42+00:00</t>
+        </is>
+      </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/PostHog/posthog/releases</t>
+          <t>https://github.com/PostHog/posthog/releases/tag/desktop-v0.61.126</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
@@ -1908,13 +1936,17 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr"/>
+          <t>agent-skills-v0.873.0</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04T08:27:02+00:00</t>
+        </is>
+      </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/PostHog/posthog/releases</t>
+          <t>https://github.com/PostHog/posthog/releases/tag/agent-skills-v0.873.0</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -1941,13 +1973,17 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr"/>
+          <t>agent-skills-v0.1559.0</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17T08:50:46+00:00</t>
+        </is>
+      </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/PostHog/posthog/releases</t>
+          <t>https://github.com/PostHog/posthog/releases/tag/agent-skills-v0.1559.0</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
@@ -1974,13 +2010,17 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr"/>
+          <t>agent-skills-v0.2010.0</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24T16:57:41+00:00</t>
+        </is>
+      </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/PostHog/posthog/releases</t>
+          <t>https://github.com/PostHog/posthog/releases/tag/agent-skills-v0.2010.0</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
@@ -6447,13 +6487,17 @@
       </c>
       <c r="G162" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H162" s="3" t="inlineStr"/>
+          <t>v0.1.1</t>
+        </is>
+      </c>
+      <c r="H162" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-10T16:58:17+00:00</t>
+        </is>
+      </c>
       <c r="I162" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/vectorize-io/hindsight/releases</t>
+          <t>https://github.com/vectorize-io/hindsight/releases/tag/v0.1.1</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr"/>
@@ -6480,13 +6524,17 @@
       </c>
       <c r="G163" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H163" s="3" t="inlineStr"/>
+          <t>v0.2.1</t>
+        </is>
+      </c>
+      <c r="H163" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-05T12:00:12+00:00</t>
+        </is>
+      </c>
       <c r="I163" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/vectorize-io/hindsight/releases</t>
+          <t>https://github.com/vectorize-io/hindsight/releases/tag/v0.2.1</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr"/>
@@ -6513,13 +6561,17 @@
       </c>
       <c r="G164" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H164" s="3" t="inlineStr"/>
+          <t>v0.4.2</t>
+        </is>
+      </c>
+      <c r="H164" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-29T18:03:06+00:00</t>
+        </is>
+      </c>
       <c r="I164" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/vectorize-io/hindsight/releases</t>
+          <t>https://github.com/vectorize-io/hindsight/releases/tag/v0.4.2</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr"/>
@@ -6546,13 +6598,17 @@
       </c>
       <c r="G165" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H165" s="3" t="inlineStr"/>
+          <t>v0.4.5</t>
+        </is>
+      </c>
+      <c r="H165" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-30T14:23:37+00:00</t>
+        </is>
+      </c>
       <c r="I165" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/vectorize-io/hindsight/releases</t>
+          <t>https://github.com/vectorize-io/hindsight/releases/tag/v0.4.5</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr"/>
@@ -6579,13 +6635,17 @@
       </c>
       <c r="G166" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H166" s="3" t="inlineStr"/>
+          <t>v0.9.0</t>
+        </is>
+      </c>
+      <c r="H166" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-07T16:42:26+00:00</t>
+        </is>
+      </c>
       <c r="I166" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/vectorize-io/hindsight/releases</t>
+          <t>https://github.com/vectorize-io/hindsight/releases/tag/v0.9.0</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr"/>
@@ -6612,13 +6672,17 @@
       </c>
       <c r="G167" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H167" s="3" t="inlineStr"/>
+          <t>v0.54.0</t>
+        </is>
+      </c>
+      <c r="H167" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-06T10:36:10+00:00</t>
+        </is>
+      </c>
       <c r="I167" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/microsoft/monaco-editor/releases</t>
+          <t>https://github.com/microsoft/monaco-editor/releases/tag/v0.54.0</t>
         </is>
       </c>
       <c r="J167" s="2" t="inlineStr"/>
@@ -6645,13 +6709,17 @@
       </c>
       <c r="G168" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H168" s="3" t="inlineStr"/>
+          <t>v0.55.0</t>
+        </is>
+      </c>
+      <c r="H168" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-20T15:20:15+00:00</t>
+        </is>
+      </c>
       <c r="I168" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/microsoft/monaco-editor/releases</t>
+          <t>https://github.com/microsoft/monaco-editor/releases/tag/v0.55.0</t>
         </is>
       </c>
       <c r="J168" s="2" t="inlineStr"/>
@@ -6678,13 +6746,17 @@
       </c>
       <c r="G169" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H169" s="3" t="inlineStr"/>
+          <t>v0.55.1</t>
+        </is>
+      </c>
+      <c r="H169" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-20T20:29:18+00:00</t>
+        </is>
+      </c>
       <c r="I169" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/microsoft/monaco-editor/releases</t>
+          <t>https://github.com/microsoft/monaco-editor/releases/tag/v0.55.1</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr"/>
@@ -6711,13 +6783,17 @@
       </c>
       <c r="G170" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H170" s="3" t="inlineStr"/>
+          <t>v0.56.0</t>
+        </is>
+      </c>
+      <c r="H170" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20T13:19:02+00:00</t>
+        </is>
+      </c>
       <c r="I170" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/microsoft/monaco-editor/releases</t>
+          <t>https://github.com/microsoft/monaco-editor/releases/tag/v0.56.0</t>
         </is>
       </c>
       <c r="J170" s="2" t="inlineStr"/>
@@ -6744,13 +6820,17 @@
       </c>
       <c r="G171" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H171" s="3" t="inlineStr"/>
+          <t>v0.57.0</t>
+        </is>
+      </c>
+      <c r="H171" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24T21:25:23+00:00</t>
+        </is>
+      </c>
       <c r="I171" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/microsoft/monaco-editor/releases</t>
+          <t>https://github.com/microsoft/monaco-editor/releases/tag/v0.57.0</t>
         </is>
       </c>
       <c r="J171" s="2" t="inlineStr"/>
@@ -6777,13 +6857,17 @@
       </c>
       <c r="G172" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H172" s="3" t="inlineStr"/>
+          <t>v25.12.29</t>
+        </is>
+      </c>
+      <c r="H172" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-29T00:48:35+00:00</t>
+        </is>
+      </c>
       <c r="I172" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/sxyazi/yazi/releases</t>
+          <t>https://github.com/sxyazi/yazi/releases/tag/v25.12.29</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr"/>
@@ -6810,13 +6894,17 @@
       </c>
       <c r="G173" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H173" s="3" t="inlineStr"/>
+          <t>v26.1.4</t>
+        </is>
+      </c>
+      <c r="H173" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-04T05:03:55+00:00</t>
+        </is>
+      </c>
       <c r="I173" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/sxyazi/yazi/releases</t>
+          <t>https://github.com/sxyazi/yazi/releases/tag/v26.1.4</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr"/>
@@ -6843,13 +6931,17 @@
       </c>
       <c r="G174" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H174" s="3" t="inlineStr"/>
+          <t>v26.1.22</t>
+        </is>
+      </c>
+      <c r="H174" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-22T15:57:14+00:00</t>
+        </is>
+      </c>
       <c r="I174" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/sxyazi/yazi/releases</t>
+          <t>https://github.com/sxyazi/yazi/releases/tag/v26.1.22</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr"/>
@@ -6876,13 +6968,17 @@
       </c>
       <c r="G175" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H175" s="3" t="inlineStr"/>
+          <t>v26.5.6</t>
+        </is>
+      </c>
+      <c r="H175" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-05T18:30:21+00:00</t>
+        </is>
+      </c>
       <c r="I175" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/sxyazi/yazi/releases</t>
+          <t>https://github.com/sxyazi/yazi/releases/tag/v26.5.6</t>
         </is>
       </c>
       <c r="J175" s="2" t="inlineStr"/>
@@ -6909,13 +7005,17 @@
       </c>
       <c r="G176" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H176" s="3" t="inlineStr"/>
+          <t>v26.9.1</t>
+        </is>
+      </c>
+      <c r="H176" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01T08:52:30+00:00</t>
+        </is>
+      </c>
       <c r="I176" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/sxyazi/yazi/releases</t>
+          <t>https://github.com/sxyazi/yazi/releases/tag/v26.9.1</t>
         </is>
       </c>
       <c r="J176" s="2" t="inlineStr"/>
@@ -6942,13 +7042,17 @@
       </c>
       <c r="G177" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H177" s="3" t="inlineStr"/>
+          <t>v0.25.11</t>
+        </is>
+      </c>
+      <c r="H177" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-15T02:13:49+00:00</t>
+        </is>
+      </c>
       <c r="I177" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/evanw/esbuild/releases</t>
+          <t>https://github.com/evanw/esbuild/releases/tag/v0.25.11</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr"/>
@@ -6975,13 +7079,17 @@
       </c>
       <c r="G178" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H178" s="3" t="inlineStr"/>
+          <t>v0.27.0</t>
+        </is>
+      </c>
+      <c r="H178" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-09T19:02:27+00:00</t>
+        </is>
+      </c>
       <c r="I178" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/evanw/esbuild/releases</t>
+          <t>https://github.com/evanw/esbuild/releases/tag/v0.27.0</t>
         </is>
       </c>
       <c r="J178" s="2" t="inlineStr"/>
@@ -7008,13 +7116,17 @@
       </c>
       <c r="G179" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H179" s="3" t="inlineStr"/>
+          <t>v0.27.1</t>
+        </is>
+      </c>
+      <c r="H179" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-03T20:25:19+00:00</t>
+        </is>
+      </c>
       <c r="I179" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/evanw/esbuild/releases</t>
+          <t>https://github.com/evanw/esbuild/releases/tag/v0.27.1</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr"/>
@@ -7041,13 +7153,17 @@
       </c>
       <c r="G180" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H180" s="3" t="inlineStr"/>
+          <t>v0.27.2</t>
+        </is>
+      </c>
+      <c r="H180" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-17T01:05:56+00:00</t>
+        </is>
+      </c>
       <c r="I180" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/evanw/esbuild/releases</t>
+          <t>https://github.com/evanw/esbuild/releases/tag/v0.27.2</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr"/>
@@ -7074,13 +7190,17 @@
       </c>
       <c r="G181" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H181" s="3" t="inlineStr"/>
+          <t>v0.27.7</t>
+        </is>
+      </c>
+      <c r="H181" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-02T16:43:53+00:00</t>
+        </is>
+      </c>
       <c r="I181" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/evanw/esbuild/releases</t>
+          <t>https://github.com/evanw/esbuild/releases/tag/v0.27.7</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr"/>
@@ -7107,13 +7227,17 @@
       </c>
       <c r="G182" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H182" s="3" t="inlineStr"/>
+          <t>v2.33.0</t>
+        </is>
+      </c>
+      <c r="H182" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-25T16:38:25+00:00</t>
+        </is>
+      </c>
       <c r="I182" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/psf/requests/releases</t>
+          <t>https://github.com/psf/requests/releases/tag/v2.33.0</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr"/>
@@ -7140,13 +7264,17 @@
       </c>
       <c r="G183" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H183" s="3" t="inlineStr"/>
+          <t>v2.33.1</t>
+        </is>
+      </c>
+      <c r="H183" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-30T16:12:09+00:00</t>
+        </is>
+      </c>
       <c r="I183" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/psf/requests/releases</t>
+          <t>https://github.com/psf/requests/releases/tag/v2.33.1</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr"/>
@@ -7173,13 +7301,17 @@
       </c>
       <c r="G184" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H184" s="3" t="inlineStr"/>
+          <t>v2.34.0</t>
+        </is>
+      </c>
+      <c r="H184" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-11T19:40:27+00:00</t>
+        </is>
+      </c>
       <c r="I184" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/psf/requests/releases</t>
+          <t>https://github.com/psf/requests/releases/tag/v2.34.0</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr"/>
@@ -7206,13 +7338,17 @@
       </c>
       <c r="G185" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H185" s="3" t="inlineStr"/>
+          <t>v2.34.1</t>
+        </is>
+      </c>
+      <c r="H185" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:23:51+00:00</t>
+        </is>
+      </c>
       <c r="I185" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/psf/requests/releases</t>
+          <t>https://github.com/psf/requests/releases/tag/v2.34.1</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr"/>
@@ -7239,13 +7375,17 @@
       </c>
       <c r="G186" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H186" s="3" t="inlineStr"/>
+          <t>v2.34.2</t>
+        </is>
+      </c>
+      <c r="H186" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14T19:27:15+00:00</t>
+        </is>
+      </c>
       <c r="I186" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/psf/requests/releases</t>
+          <t>https://github.com/psf/requests/releases/tag/v2.34.2</t>
         </is>
       </c>
       <c r="J186" s="2" t="inlineStr"/>
@@ -7272,13 +7412,17 @@
       </c>
       <c r="G187" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H187" s="3" t="inlineStr"/>
+          <t>v4.1.14</t>
+        </is>
+      </c>
+      <c r="H187" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-01T16:00:08+00:00</t>
+        </is>
+      </c>
       <c r="I187" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/tailwindlabs/tailwindcss/releases</t>
+          <t>https://github.com/tailwindlabs/tailwindcss/releases/tag/v4.1.14</t>
         </is>
       </c>
       <c r="J187" s="2" t="inlineStr"/>
@@ -7305,13 +7449,17 @@
       </c>
       <c r="G188" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H188" s="3" t="inlineStr"/>
+          <t>v4.1.16</t>
+        </is>
+      </c>
+      <c r="H188" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-23T10:55:20+00:00</t>
+        </is>
+      </c>
       <c r="I188" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/tailwindlabs/tailwindcss/releases</t>
+          <t>https://github.com/tailwindlabs/tailwindcss/releases/tag/v4.1.16</t>
         </is>
       </c>
       <c r="J188" s="2" t="inlineStr"/>
@@ -7338,13 +7486,17 @@
       </c>
       <c r="G189" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H189" s="3" t="inlineStr"/>
+          <t>v4.2.1</t>
+        </is>
+      </c>
+      <c r="H189" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-23T12:51:32+00:00</t>
+        </is>
+      </c>
       <c r="I189" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/tailwindlabs/tailwindcss/releases</t>
+          <t>https://github.com/tailwindlabs/tailwindcss/releases/tag/v4.2.1</t>
         </is>
       </c>
       <c r="J189" s="2" t="inlineStr"/>
@@ -7371,13 +7523,17 @@
       </c>
       <c r="G190" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H190" s="3" t="inlineStr"/>
+          <t>v4.2.2</t>
+        </is>
+      </c>
+      <c r="H190" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-18T16:06:04+00:00</t>
+        </is>
+      </c>
       <c r="I190" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/tailwindlabs/tailwindcss/releases</t>
+          <t>https://github.com/tailwindlabs/tailwindcss/releases/tag/v4.2.2</t>
         </is>
       </c>
       <c r="J190" s="2" t="inlineStr"/>
@@ -7404,13 +7560,17 @@
       </c>
       <c r="G191" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H191" s="3" t="inlineStr"/>
+          <t>v4.3.2</t>
+        </is>
+      </c>
+      <c r="H191" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29T14:21:45+00:00</t>
+        </is>
+      </c>
       <c r="I191" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/tailwindlabs/tailwindcss/releases</t>
+          <t>https://github.com/tailwindlabs/tailwindcss/releases/tag/v4.3.2</t>
         </is>
       </c>
       <c r="J191" s="2" t="inlineStr"/>
@@ -7437,13 +7597,17 @@
       </c>
       <c r="G192" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H192" s="3" t="inlineStr"/>
+          <t>v40.1.0</t>
+        </is>
+      </c>
+      <c r="H192" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-29T02:25:36+00:00</t>
+        </is>
+      </c>
       <c r="I192" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/electron/electron/releases</t>
+          <t>https://github.com/electron/electron/releases/tag/v40.1.0</t>
         </is>
       </c>
       <c r="J192" s="2" t="inlineStr"/>
@@ -7470,13 +7634,17 @@
       </c>
       <c r="G193" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H193" s="3" t="inlineStr"/>
+          <t>v42.4.0</t>
+        </is>
+      </c>
+      <c r="H193" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09T08:30:31+00:00</t>
+        </is>
+      </c>
       <c r="I193" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/electron/electron/releases</t>
+          <t>https://github.com/electron/electron/releases/tag/v42.4.0</t>
         </is>
       </c>
       <c r="J193" s="2" t="inlineStr"/>
@@ -7503,13 +7671,17 @@
       </c>
       <c r="G194" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H194" s="3" t="inlineStr"/>
+          <t>v41.10.6</t>
+        </is>
+      </c>
+      <c r="H194" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-18T18:28:23+00:00</t>
+        </is>
+      </c>
       <c r="I194" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/electron/electron/releases</t>
+          <t>https://github.com/electron/electron/releases/tag/v41.10.6</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr"/>
@@ -7536,13 +7708,17 @@
       </c>
       <c r="G195" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H195" s="3" t="inlineStr"/>
+          <t>v43.5.1</t>
+        </is>
+      </c>
+      <c r="H195" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01T18:11:42+00:00</t>
+        </is>
+      </c>
       <c r="I195" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/electron/electron/releases</t>
+          <t>https://github.com/electron/electron/releases/tag/v43.5.1</t>
         </is>
       </c>
       <c r="J195" s="2" t="inlineStr"/>
@@ -7569,13 +7745,17 @@
       </c>
       <c r="G196" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H196" s="3" t="inlineStr"/>
+          <t>v42.11.8</t>
+        </is>
+      </c>
+      <c r="H196" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-23T06:37:29+00:00</t>
+        </is>
+      </c>
       <c r="I196" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/electron/electron/releases</t>
+          <t>https://github.com/electron/electron/releases/tag/v42.11.8</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr"/>
@@ -7602,13 +7782,17 @@
       </c>
       <c r="G197" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H197" s="3" t="inlineStr"/>
+          <t>bun-v1.3.12</t>
+        </is>
+      </c>
+      <c r="H197" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-10T03:04:46+00:00</t>
+        </is>
+      </c>
       <c r="I197" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/oven-sh/bun/releases</t>
+          <t>https://github.com/oven-sh/bun/releases/tag/bun-v1.3.12</t>
         </is>
       </c>
       <c r="J197" s="2" t="inlineStr"/>
@@ -7635,13 +7819,17 @@
       </c>
       <c r="G198" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H198" s="3" t="inlineStr"/>
+          <t>bun-v1.3.13</t>
+        </is>
+      </c>
+      <c r="H198" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-20T08:07:57+00:00</t>
+        </is>
+      </c>
       <c r="I198" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/oven-sh/bun/releases</t>
+          <t>https://github.com/oven-sh/bun/releases/tag/bun-v1.3.13</t>
         </is>
       </c>
       <c r="J198" s="2" t="inlineStr"/>
@@ -7668,13 +7856,17 @@
       </c>
       <c r="G199" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H199" s="3" t="inlineStr"/>
+          <t>bun-v1.3.14</t>
+        </is>
+      </c>
+      <c r="H199" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13T03:48:28+00:00</t>
+        </is>
+      </c>
       <c r="I199" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/oven-sh/bun/releases</t>
+          <t>https://github.com/oven-sh/bun/releases/tag/bun-v1.3.14</t>
         </is>
       </c>
       <c r="J199" s="2" t="inlineStr"/>
@@ -7701,13 +7893,17 @@
       </c>
       <c r="G200" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H200" s="3" t="inlineStr"/>
+          <t>bun-v1.4.0</t>
+        </is>
+      </c>
+      <c r="H200" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-20T14:07:21+00:00</t>
+        </is>
+      </c>
       <c r="I200" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/oven-sh/bun/releases</t>
+          <t>https://github.com/oven-sh/bun/releases/tag/bun-v1.4.0</t>
         </is>
       </c>
       <c r="J200" s="2" t="inlineStr"/>
@@ -7734,13 +7930,17 @@
       </c>
       <c r="G201" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H201" s="3" t="inlineStr"/>
+          <t>bun-v1.4.1</t>
+        </is>
+      </c>
+      <c r="H201" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-04T08:33:19+00:00</t>
+        </is>
+      </c>
       <c r="I201" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/oven-sh/bun/releases</t>
+          <t>https://github.com/oven-sh/bun/releases/tag/bun-v1.4.1</t>
         </is>
       </c>
       <c r="J201" s="2" t="inlineStr"/>
@@ -7767,13 +7967,17 @@
       </c>
       <c r="G202" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H202" s="3" t="inlineStr"/>
+          <t>v10.11.3</t>
+        </is>
+      </c>
+      <c r="H202" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-16T22:40:10+00:00</t>
+        </is>
+      </c>
       <c r="I202" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/jellyfin/jellyfin/releases</t>
+          <t>https://github.com/jellyfin/jellyfin/releases/tag/v10.11.3</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr"/>
@@ -7800,13 +8004,17 @@
       </c>
       <c r="G203" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H203" s="3" t="inlineStr"/>
+          <t>v10.11.4</t>
+        </is>
+      </c>
+      <c r="H203" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-01T02:33:37+00:00</t>
+        </is>
+      </c>
       <c r="I203" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/jellyfin/jellyfin/releases</t>
+          <t>https://github.com/jellyfin/jellyfin/releases/tag/v10.11.4</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr"/>
@@ -7833,13 +8041,17 @@
       </c>
       <c r="G204" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H204" s="3" t="inlineStr"/>
+          <t>v10.11.9</t>
+        </is>
+      </c>
+      <c r="H204" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21T01:59:59+00:00</t>
+        </is>
+      </c>
       <c r="I204" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/jellyfin/jellyfin/releases</t>
+          <t>https://github.com/jellyfin/jellyfin/releases/tag/v10.11.9</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr"/>
@@ -7866,13 +8078,17 @@
       </c>
       <c r="G205" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H205" s="3" t="inlineStr"/>
+          <t>v10.11.11</t>
+        </is>
+      </c>
+      <c r="H205" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-06T16:18:54+00:00</t>
+        </is>
+      </c>
       <c r="I205" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/jellyfin/jellyfin/releases</t>
+          <t>https://github.com/jellyfin/jellyfin/releases/tag/v10.11.11</t>
         </is>
       </c>
       <c r="J205" s="2" t="inlineStr"/>
@@ -7899,13 +8115,17 @@
       </c>
       <c r="G206" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H206" s="3" t="inlineStr"/>
+          <t>v12.0</t>
+        </is>
+      </c>
+      <c r="H206" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08T01:38:39+00:00</t>
+        </is>
+      </c>
       <c r="I206" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/jellyfin/jellyfin/releases</t>
+          <t>https://github.com/jellyfin/jellyfin/releases/tag/v12.0</t>
         </is>
       </c>
       <c r="J206" s="2" t="inlineStr"/>
@@ -7932,13 +8152,17 @@
       </c>
       <c r="G207" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H207" s="3" t="inlineStr"/>
+          <t>v10.3.1</t>
+        </is>
+      </c>
+      <c r="H207" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-20T15:26:41+00:00</t>
+        </is>
+      </c>
       <c r="I207" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/schollz/croc/releases</t>
+          <t>https://github.com/schollz/croc/releases/tag/v10.3.1</t>
         </is>
       </c>
       <c r="J207" s="2" t="inlineStr"/>
@@ -7965,13 +8189,17 @@
       </c>
       <c r="G208" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H208" s="3" t="inlineStr"/>
+          <t>v11.1.1</t>
+        </is>
+      </c>
+      <c r="H208" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-15T21:21:47+00:00</t>
+        </is>
+      </c>
       <c r="I208" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/schollz/croc/releases</t>
+          <t>https://github.com/schollz/croc/releases/tag/v11.1.1</t>
         </is>
       </c>
       <c r="J208" s="2" t="inlineStr"/>
@@ -7998,13 +8226,17 @@
       </c>
       <c r="G209" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H209" s="3" t="inlineStr"/>
+          <t>v11.3.1</t>
+        </is>
+      </c>
+      <c r="H209" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25T09:17:08+00:00</t>
+        </is>
+      </c>
       <c r="I209" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/schollz/croc/releases</t>
+          <t>https://github.com/schollz/croc/releases/tag/v11.3.1</t>
         </is>
       </c>
       <c r="J209" s="2" t="inlineStr"/>
@@ -8031,13 +8263,17 @@
       </c>
       <c r="G210" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H210" s="3" t="inlineStr"/>
+          <t>v11.5.1</t>
+        </is>
+      </c>
+      <c r="H210" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:49:07+00:00</t>
+        </is>
+      </c>
       <c r="I210" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/schollz/croc/releases</t>
+          <t>https://github.com/schollz/croc/releases/tag/v11.5.1</t>
         </is>
       </c>
       <c r="J210" s="2" t="inlineStr"/>
@@ -8064,13 +8300,17 @@
       </c>
       <c r="G211" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H211" s="3" t="inlineStr"/>
+          <t>v11.5.4</t>
+        </is>
+      </c>
+      <c r="H211" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-26T21:53:50+00:00</t>
+        </is>
+      </c>
       <c r="I211" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/schollz/croc/releases</t>
+          <t>https://github.com/schollz/croc/releases/tag/v11.5.4</t>
         </is>
       </c>
       <c r="J211" s="2" t="inlineStr"/>
@@ -8097,13 +8337,17 @@
       </c>
       <c r="G212" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H212" s="3" t="inlineStr"/>
+          <t>v7.5.5</t>
+        </is>
+      </c>
+      <c r="H212" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-12T18:19:38+00:00</t>
+        </is>
+      </c>
       <c r="I212" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/PowerShell/PowerShell/releases</t>
+          <t>https://github.com/PowerShell/PowerShell/releases/tag/v7.5.5</t>
         </is>
       </c>
       <c r="J212" s="2" t="inlineStr"/>
@@ -8130,13 +8374,17 @@
       </c>
       <c r="G213" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H213" s="3" t="inlineStr"/>
+          <t>v7.5.6</t>
+        </is>
+      </c>
+      <c r="H213" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-21T19:08:26+00:00</t>
+        </is>
+      </c>
       <c r="I213" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/PowerShell/PowerShell/releases</t>
+          <t>https://github.com/PowerShell/PowerShell/releases/tag/v7.5.6</t>
         </is>
       </c>
       <c r="J213" s="2" t="inlineStr"/>
@@ -8163,13 +8411,17 @@
       </c>
       <c r="G214" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H214" s="3" t="inlineStr"/>
+          <t>v7.4.16</t>
+        </is>
+      </c>
+      <c r="H214" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21T20:42:02+00:00</t>
+        </is>
+      </c>
       <c r="I214" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/PowerShell/PowerShell/releases</t>
+          <t>https://github.com/PowerShell/PowerShell/releases/tag/v7.4.16</t>
         </is>
       </c>
       <c r="J214" s="2" t="inlineStr"/>
@@ -8196,13 +8448,17 @@
       </c>
       <c r="G215" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H215" s="3" t="inlineStr"/>
+          <t>v7.5.11</t>
+        </is>
+      </c>
+      <c r="H215" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08T20:25:50+00:00</t>
+        </is>
+      </c>
       <c r="I215" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/PowerShell/PowerShell/releases</t>
+          <t>https://github.com/PowerShell/PowerShell/releases/tag/v7.5.11</t>
         </is>
       </c>
       <c r="J215" s="2" t="inlineStr"/>
@@ -8229,13 +8485,17 @@
       </c>
       <c r="G216" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H216" s="3" t="inlineStr"/>
+          <t>v7.4.20</t>
+        </is>
+      </c>
+      <c r="H216" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08T21:09:53+00:00</t>
+        </is>
+      </c>
       <c r="I216" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/PowerShell/PowerShell/releases</t>
+          <t>https://github.com/PowerShell/PowerShell/releases/tag/v7.4.20</t>
         </is>
       </c>
       <c r="J216" s="2" t="inlineStr"/>
@@ -8262,13 +8522,17 @@
       </c>
       <c r="G217" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H217" s="3" t="inlineStr"/>
+          <t>v1.2.0</t>
+        </is>
+      </c>
+      <c r="H217" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-07T16:29:37+00:00</t>
+        </is>
+      </c>
       <c r="I217" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/career-ops-hq/career-ops/releases</t>
+          <t>https://github.com/career-ops-hq/career-ops/releases/tag/v1.2.0</t>
         </is>
       </c>
       <c r="J217" s="2" t="inlineStr"/>
@@ -8295,13 +8559,17 @@
       </c>
       <c r="G218" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H218" s="3" t="inlineStr"/>
+          <t>v1.5.0</t>
+        </is>
+      </c>
+      <c r="H218" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-14T17:34:23+00:00</t>
+        </is>
+      </c>
       <c r="I218" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/career-ops-hq/career-ops/releases</t>
+          <t>https://github.com/career-ops-hq/career-ops/releases/tag/v1.5.0</t>
         </is>
       </c>
       <c r="J218" s="2" t="inlineStr"/>
@@ -8328,13 +8596,17 @@
       </c>
       <c r="G219" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H219" s="3" t="inlineStr"/>
+          <t>career-ops-v1.7.1</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-12T17:27:44+00:00</t>
+        </is>
+      </c>
       <c r="I219" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/career-ops-hq/career-ops/releases</t>
+          <t>https://github.com/career-ops-hq/career-ops/releases/tag/career-ops-v1.7.1</t>
         </is>
       </c>
       <c r="J219" s="2" t="inlineStr"/>
@@ -8361,13 +8633,17 @@
       </c>
       <c r="G220" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H220" s="3" t="inlineStr"/>
+          <t>career-ops-v1.20.0</t>
+        </is>
+      </c>
+      <c r="H220" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14T20:06:58+00:00</t>
+        </is>
+      </c>
       <c r="I220" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/career-ops-hq/career-ops/releases</t>
+          <t>https://github.com/career-ops-hq/career-ops/releases/tag/career-ops-v1.20.0</t>
         </is>
       </c>
       <c r="J220" s="2" t="inlineStr"/>
@@ -8394,13 +8670,17 @@
       </c>
       <c r="G221" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H221" s="3" t="inlineStr"/>
+          <t>web-v0.6.1</t>
+        </is>
+      </c>
+      <c r="H221" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10T22:06:57+00:00</t>
+        </is>
+      </c>
       <c r="I221" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/career-ops-hq/career-ops/releases</t>
+          <t>https://github.com/career-ops-hq/career-ops/releases/tag/web-v0.6.1</t>
         </is>
       </c>
       <c r="J221" s="2" t="inlineStr"/>
@@ -8427,13 +8707,17 @@
       </c>
       <c r="G222" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H222" s="3" t="inlineStr"/>
+          <t>v1.11.0</t>
+        </is>
+      </c>
+      <c r="H222" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-12T08:01:16+00:00</t>
+        </is>
+      </c>
       <c r="I222" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/gkd-kit/gkd/releases</t>
+          <t>https://github.com/gkd-kit/gkd/releases/tag/v1.11.0</t>
         </is>
       </c>
       <c r="J222" s="2" t="inlineStr"/>
@@ -8460,13 +8744,17 @@
       </c>
       <c r="G223" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H223" s="3" t="inlineStr"/>
+          <t>v1.11.1</t>
+        </is>
+      </c>
+      <c r="H223" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-13T11:46:28+00:00</t>
+        </is>
+      </c>
       <c r="I223" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/gkd-kit/gkd/releases</t>
+          <t>https://github.com/gkd-kit/gkd/releases/tag/v1.11.1</t>
         </is>
       </c>
       <c r="J223" s="2" t="inlineStr"/>
@@ -8493,13 +8781,17 @@
       </c>
       <c r="G224" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H224" s="3" t="inlineStr"/>
+          <t>v1.11.3</t>
+        </is>
+      </c>
+      <c r="H224" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-17T07:54:08+00:00</t>
+        </is>
+      </c>
       <c r="I224" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/gkd-kit/gkd/releases</t>
+          <t>https://github.com/gkd-kit/gkd/releases/tag/v1.11.3</t>
         </is>
       </c>
       <c r="J224" s="2" t="inlineStr"/>
@@ -8526,13 +8818,17 @@
       </c>
       <c r="G225" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H225" s="3" t="inlineStr"/>
+          <t>v1.11.4</t>
+        </is>
+      </c>
+      <c r="H225" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-20T11:17:33+00:00</t>
+        </is>
+      </c>
       <c r="I225" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/gkd-kit/gkd/releases</t>
+          <t>https://github.com/gkd-kit/gkd/releases/tag/v1.11.4</t>
         </is>
       </c>
       <c r="J225" s="2" t="inlineStr"/>
@@ -8559,13 +8855,17 @@
       </c>
       <c r="G226" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H226" s="3" t="inlineStr"/>
+          <t>v1.11.6</t>
+        </is>
+      </c>
+      <c r="H226" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-13T18:03:36+00:00</t>
+        </is>
+      </c>
       <c r="I226" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/gkd-kit/gkd/releases</t>
+          <t>https://github.com/gkd-kit/gkd/releases/tag/v1.11.6</t>
         </is>
       </c>
       <c r="J226" s="2" t="inlineStr"/>
@@ -8592,13 +8892,17 @@
       </c>
       <c r="G227" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H227" s="3" t="inlineStr"/>
+          <t>v1.23.13503.0</t>
+        </is>
+      </c>
+      <c r="H227" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-17T23:42:36+00:00</t>
+        </is>
+      </c>
       <c r="I227" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/microsoft/terminal/releases</t>
+          <t>https://github.com/microsoft/terminal/releases/tag/v1.23.13503.0</t>
         </is>
       </c>
       <c r="J227" s="2" t="inlineStr"/>
@@ -8625,13 +8929,17 @@
       </c>
       <c r="G228" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H228" s="3" t="inlineStr"/>
+          <t>v1.23.20211.0</t>
+        </is>
+      </c>
+      <c r="H228" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-24T00:01:18+00:00</t>
+        </is>
+      </c>
       <c r="I228" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/microsoft/terminal/releases</t>
+          <t>https://github.com/microsoft/terminal/releases/tag/v1.23.20211.0</t>
         </is>
       </c>
       <c r="J228" s="2" t="inlineStr"/>
@@ -8658,13 +8966,17 @@
       </c>
       <c r="G229" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H229" s="3" t="inlineStr"/>
+          <t>v1.24.10921.0</t>
+        </is>
+      </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-03T23:39:36+00:00</t>
+        </is>
+      </c>
       <c r="I229" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/microsoft/terminal/releases</t>
+          <t>https://github.com/microsoft/terminal/releases/tag/v1.24.10921.0</t>
         </is>
       </c>
       <c r="J229" s="2" t="inlineStr"/>
@@ -8691,13 +9003,17 @@
       </c>
       <c r="G230" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H230" s="3" t="inlineStr"/>
+          <t>v1.24.11321.0</t>
+        </is>
+      </c>
+      <c r="H230" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13T21:14:56+00:00</t>
+        </is>
+      </c>
       <c r="I230" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/microsoft/terminal/releases</t>
+          <t>https://github.com/microsoft/terminal/releases/tag/v1.24.11321.0</t>
         </is>
       </c>
       <c r="J230" s="2" t="inlineStr"/>
@@ -8724,13 +9040,17 @@
       </c>
       <c r="G231" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H231" s="3" t="inlineStr"/>
+          <t>v1.24.11911.0</t>
+        </is>
+      </c>
+      <c r="H231" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16T21:56:12+00:00</t>
+        </is>
+      </c>
       <c r="I231" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/microsoft/terminal/releases</t>
+          <t>https://github.com/microsoft/terminal/releases/tag/v1.24.11911.0</t>
         </is>
       </c>
       <c r="J231" s="2" t="inlineStr"/>
@@ -8757,13 +9077,17 @@
       </c>
       <c r="G232" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H232" s="3" t="inlineStr"/>
+          <t>v2.8.7</t>
+        </is>
+      </c>
+      <c r="H232" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-05T18:01:37+00:00</t>
+        </is>
+      </c>
       <c r="I232" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/MHSanaei/3x-ui/releases</t>
+          <t>https://github.com/MHSanaei/3x-ui/releases/tag/v2.8.7</t>
         </is>
       </c>
       <c r="J232" s="2" t="inlineStr"/>
@@ -8790,13 +9114,17 @@
       </c>
       <c r="G233" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H233" s="3" t="inlineStr"/>
+          <t>v3.2.5</t>
+        </is>
+      </c>
+      <c r="H233" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01T08:34:01+00:00</t>
+        </is>
+      </c>
       <c r="I233" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/MHSanaei/3x-ui/releases</t>
+          <t>https://github.com/MHSanaei/3x-ui/releases/tag/v3.2.5</t>
         </is>
       </c>
       <c r="J233" s="2" t="inlineStr"/>
@@ -8823,13 +9151,17 @@
       </c>
       <c r="G234" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H234" s="3" t="inlineStr"/>
+          <t>v3.2.6</t>
+        </is>
+      </c>
+      <c r="H234" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02T02:24:02+00:00</t>
+        </is>
+      </c>
       <c r="I234" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/MHSanaei/3x-ui/releases</t>
+          <t>https://github.com/MHSanaei/3x-ui/releases/tag/v3.2.6</t>
         </is>
       </c>
       <c r="J234" s="2" t="inlineStr"/>
@@ -8856,13 +9188,17 @@
       </c>
       <c r="G235" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H235" s="3" t="inlineStr"/>
+          <t>v3.2.8</t>
+        </is>
+      </c>
+      <c r="H235" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05T09:11:57+00:00</t>
+        </is>
+      </c>
       <c r="I235" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/MHSanaei/3x-ui/releases</t>
+          <t>https://github.com/MHSanaei/3x-ui/releases/tag/v3.2.8</t>
         </is>
       </c>
       <c r="J235" s="2" t="inlineStr"/>
@@ -8889,13 +9225,17 @@
       </c>
       <c r="G236" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H236" s="3" t="inlineStr"/>
+          <t>v3.4.1</t>
+        </is>
+      </c>
+      <c r="H236" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25T22:54:29+00:00</t>
+        </is>
+      </c>
       <c r="I236" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/MHSanaei/3x-ui/releases</t>
+          <t>https://github.com/MHSanaei/3x-ui/releases/tag/v3.4.1</t>
         </is>
       </c>
       <c r="J236" s="2" t="inlineStr"/>
@@ -8922,13 +9262,17 @@
       </c>
       <c r="G237" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H237" s="3" t="inlineStr"/>
+          <t>v7.0.0</t>
+        </is>
+      </c>
+      <c r="H237" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-08T08:05:43+00:00</t>
+        </is>
+      </c>
       <c r="I237" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/vadimdemedes/ink/releases</t>
+          <t>https://github.com/vadimdemedes/ink/releases/tag/v7.0.0</t>
         </is>
       </c>
       <c r="J237" s="2" t="inlineStr"/>
@@ -8955,13 +9299,17 @@
       </c>
       <c r="G238" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H238" s="3" t="inlineStr"/>
+          <t>v7.0.2</t>
+        </is>
+      </c>
+      <c r="H238" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-05T09:17:55+00:00</t>
+        </is>
+      </c>
       <c r="I238" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/vadimdemedes/ink/releases</t>
+          <t>https://github.com/vadimdemedes/ink/releases/tag/v7.0.2</t>
         </is>
       </c>
       <c r="J238" s="2" t="inlineStr"/>
@@ -8988,13 +9336,17 @@
       </c>
       <c r="G239" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H239" s="3" t="inlineStr"/>
+          <t>v7.0.4</t>
+        </is>
+      </c>
+      <c r="H239" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-24T17:10:01+00:00</t>
+        </is>
+      </c>
       <c r="I239" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/vadimdemedes/ink/releases</t>
+          <t>https://github.com/vadimdemedes/ink/releases/tag/v7.0.4</t>
         </is>
       </c>
       <c r="J239" s="2" t="inlineStr"/>
@@ -9021,13 +9373,17 @@
       </c>
       <c r="G240" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H240" s="3" t="inlineStr"/>
+          <t>v7.0.5</t>
+        </is>
+      </c>
+      <c r="H240" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29T21:15:50+00:00</t>
+        </is>
+      </c>
       <c r="I240" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/vadimdemedes/ink/releases</t>
+          <t>https://github.com/vadimdemedes/ink/releases/tag/v7.0.5</t>
         </is>
       </c>
       <c r="J240" s="2" t="inlineStr"/>
@@ -9054,13 +9410,17 @@
       </c>
       <c r="G241" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H241" s="3" t="inlineStr"/>
+          <t>v7.0.6</t>
+        </is>
+      </c>
+      <c r="H241" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12T23:37:17+00:00</t>
+        </is>
+      </c>
       <c r="I241" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/vadimdemedes/ink/releases</t>
+          <t>https://github.com/vadimdemedes/ink/releases/tag/v7.0.6</t>
         </is>
       </c>
       <c r="J241" s="2" t="inlineStr"/>
@@ -9087,13 +9447,17 @@
       </c>
       <c r="G242" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H242" s="3" t="inlineStr"/>
+          <t>v0.25.2</t>
+        </is>
+      </c>
+      <c r="H242" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-24T12:30:04+00:00</t>
+        </is>
+      </c>
       <c r="I242" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/usememos/memos/releases</t>
+          <t>https://github.com/usememos/memos/releases/tag/v0.25.2</t>
         </is>
       </c>
       <c r="J242" s="2" t="inlineStr"/>
@@ -9120,13 +9484,17 @@
       </c>
       <c r="G243" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H243" s="3" t="inlineStr"/>
+          <t>v0.25.3</t>
+        </is>
+      </c>
+      <c r="H243" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-25T15:40:41+00:00</t>
+        </is>
+      </c>
       <c r="I243" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/usememos/memos/releases</t>
+          <t>https://github.com/usememos/memos/releases/tag/v0.25.3</t>
         </is>
       </c>
       <c r="J243" s="2" t="inlineStr"/>
@@ -9153,13 +9521,17 @@
       </c>
       <c r="G244" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H244" s="3" t="inlineStr"/>
+          <t>v0.26.0</t>
+        </is>
+      </c>
+      <c r="H244" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-31T15:28:09+00:00</t>
+        </is>
+      </c>
       <c r="I244" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/usememos/memos/releases</t>
+          <t>https://github.com/usememos/memos/releases/tag/v0.26.0</t>
         </is>
       </c>
       <c r="J244" s="2" t="inlineStr"/>
@@ -9186,13 +9558,17 @@
       </c>
       <c r="G245" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H245" s="3" t="inlineStr"/>
+          <t>v0.27.0</t>
+        </is>
+      </c>
+      <c r="H245" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-18T20:03:07+00:00</t>
+        </is>
+      </c>
       <c r="I245" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/usememos/memos/releases</t>
+          <t>https://github.com/usememos/memos/releases/tag/v0.27.0</t>
         </is>
       </c>
       <c r="J245" s="2" t="inlineStr"/>
@@ -9219,13 +9595,17 @@
       </c>
       <c r="G246" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H246" s="3" t="inlineStr"/>
+          <t>v0.30.0</t>
+        </is>
+      </c>
+      <c r="H246" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-26T15:46:00+00:00</t>
+        </is>
+      </c>
       <c r="I246" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/usememos/memos/releases</t>
+          <t>https://github.com/usememos/memos/releases/tag/v0.30.0</t>
         </is>
       </c>
       <c r="J246" s="2" t="inlineStr"/>
@@ -9252,13 +9632,17 @@
       </c>
       <c r="G247" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H247" s="3" t="inlineStr"/>
+          <t>v4.0.0-beta.437</t>
+        </is>
+      </c>
+      <c r="H247" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-21T07:12:25+00:00</t>
+        </is>
+      </c>
       <c r="I247" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/coollabsio/coolify/releases</t>
+          <t>https://github.com/coollabsio/coolify/releases/tag/v4.0.0-beta.437</t>
         </is>
       </c>
       <c r="J247" s="2" t="inlineStr"/>
@@ -9285,13 +9669,17 @@
       </c>
       <c r="G248" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H248" s="3" t="inlineStr"/>
+          <t>v4.0.0-beta.468</t>
+        </is>
+      </c>
+      <c r="H248" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-12T13:28:09+00:00</t>
+        </is>
+      </c>
       <c r="I248" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/coollabsio/coolify/releases</t>
+          <t>https://github.com/coollabsio/coolify/releases/tag/v4.0.0-beta.468</t>
         </is>
       </c>
       <c r="J248" s="2" t="inlineStr"/>
@@ -9318,13 +9706,17 @@
       </c>
       <c r="G249" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H249" s="3" t="inlineStr"/>
+          <t>v4.3.0</t>
+        </is>
+      </c>
+      <c r="H249" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-12T10:04:38+00:00</t>
+        </is>
+      </c>
       <c r="I249" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/coollabsio/coolify/releases</t>
+          <t>https://github.com/coollabsio/coolify/releases/tag/v4.3.0</t>
         </is>
       </c>
       <c r="J249" s="2" t="inlineStr"/>
@@ -9351,13 +9743,17 @@
       </c>
       <c r="G250" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H250" s="3" t="inlineStr"/>
+          <t>v4.3.5</t>
+        </is>
+      </c>
+      <c r="H250" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-16T11:59:45+00:00</t>
+        </is>
+      </c>
       <c r="I250" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/coollabsio/coolify/releases</t>
+          <t>https://github.com/coollabsio/coolify/releases/tag/v4.3.5</t>
         </is>
       </c>
       <c r="J250" s="2" t="inlineStr"/>
@@ -9384,13 +9780,17 @@
       </c>
       <c r="G251" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H251" s="3" t="inlineStr"/>
+          <t>v4.3.21</t>
+        </is>
+      </c>
+      <c r="H251" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-15T11:41:19+00:00</t>
+        </is>
+      </c>
       <c r="I251" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/coollabsio/coolify/releases</t>
+          <t>https://github.com/coollabsio/coolify/releases/tag/v4.3.21</t>
         </is>
       </c>
       <c r="J251" s="2" t="inlineStr"/>
@@ -9417,13 +9817,17 @@
       </c>
       <c r="G252" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H252" s="3" t="inlineStr"/>
+          <t>mineru-3.0.0-released</t>
+        </is>
+      </c>
+      <c r="H252" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-28T20:13:48+00:00</t>
+        </is>
+      </c>
       <c r="I252" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/opendatalab/MinerU/releases</t>
+          <t>https://github.com/opendatalab/MinerU/releases/tag/mineru-3.0.0-released</t>
         </is>
       </c>
       <c r="J252" s="2" t="inlineStr"/>
@@ -9450,13 +9854,17 @@
       </c>
       <c r="G253" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H253" s="3" t="inlineStr"/>
+          <t>mineru-3.0.1-released</t>
+        </is>
+      </c>
+      <c r="H253" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-29T05:31:07+00:00</t>
+        </is>
+      </c>
       <c r="I253" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/opendatalab/MinerU/releases</t>
+          <t>https://github.com/opendatalab/MinerU/releases/tag/mineru-3.0.1-released</t>
         </is>
       </c>
       <c r="J253" s="2" t="inlineStr"/>
@@ -9483,13 +9891,17 @@
       </c>
       <c r="G254" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H254" s="3" t="inlineStr"/>
+          <t>mineru-3.0.6-released</t>
+        </is>
+      </c>
+      <c r="H254" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-01T12:54:58+00:00</t>
+        </is>
+      </c>
       <c r="I254" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/opendatalab/MinerU/releases</t>
+          <t>https://github.com/opendatalab/MinerU/releases/tag/mineru-3.0.6-released</t>
         </is>
       </c>
       <c r="J254" s="2" t="inlineStr"/>
@@ -9516,13 +9928,17 @@
       </c>
       <c r="G255" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H255" s="3" t="inlineStr"/>
+          <t>mineru-3.2.1-released</t>
+        </is>
+      </c>
+      <c r="H255" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-28T16:01:33+00:00</t>
+        </is>
+      </c>
       <c r="I255" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/opendatalab/MinerU/releases</t>
+          <t>https://github.com/opendatalab/MinerU/releases/tag/mineru-3.2.1-released</t>
         </is>
       </c>
       <c r="J255" s="2" t="inlineStr"/>
@@ -9549,13 +9965,17 @@
       </c>
       <c r="G256" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H256" s="3" t="inlineStr"/>
+          <t>mineru-3.3.0-released</t>
+        </is>
+      </c>
+      <c r="H256" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11T11:05:44+00:00</t>
+        </is>
+      </c>
       <c r="I256" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/opendatalab/MinerU/releases</t>
+          <t>https://github.com/opendatalab/MinerU/releases/tag/mineru-3.3.0-released</t>
         </is>
       </c>
       <c r="J256" s="2" t="inlineStr"/>
@@ -9582,13 +10002,17 @@
       </c>
       <c r="G257" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H257" s="3" t="inlineStr"/>
+          <t>v3.5.1</t>
+        </is>
+      </c>
+      <c r="H257" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-14T02:46:50+00:00</t>
+        </is>
+      </c>
       <c r="I257" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/farion1231/cc-switch/releases</t>
+          <t>https://github.com/farion1231/cc-switch/releases/tag/v3.5.1</t>
         </is>
       </c>
       <c r="J257" s="2" t="inlineStr"/>
@@ -9615,13 +10039,17 @@
       </c>
       <c r="G258" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H258" s="3" t="inlineStr"/>
+          <t>v3.18.0</t>
+        </is>
+      </c>
+      <c r="H258" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21T15:34:53+00:00</t>
+        </is>
+      </c>
       <c r="I258" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/farion1231/cc-switch/releases</t>
+          <t>https://github.com/farion1231/cc-switch/releases/tag/v3.18.0</t>
         </is>
       </c>
       <c r="J258" s="2" t="inlineStr"/>
@@ -9648,13 +10076,17 @@
       </c>
       <c r="G259" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H259" s="3" t="inlineStr"/>
+          <t>v3.19.2</t>
+        </is>
+      </c>
+      <c r="H259" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-06T04:39:34+00:00</t>
+        </is>
+      </c>
       <c r="I259" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/farion1231/cc-switch/releases</t>
+          <t>https://github.com/farion1231/cc-switch/releases/tag/v3.19.2</t>
         </is>
       </c>
       <c r="J259" s="2" t="inlineStr"/>
@@ -9681,13 +10113,17 @@
       </c>
       <c r="G260" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H260" s="3" t="inlineStr"/>
+          <t>v3.20.3</t>
+        </is>
+      </c>
+      <c r="H260" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11T16:10:52+00:00</t>
+        </is>
+      </c>
       <c r="I260" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/farion1231/cc-switch/releases</t>
+          <t>https://github.com/farion1231/cc-switch/releases/tag/v3.20.3</t>
         </is>
       </c>
       <c r="J260" s="2" t="inlineStr"/>
@@ -9714,13 +10150,17 @@
       </c>
       <c r="G261" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H261" s="3" t="inlineStr"/>
+          <t>v3.20.4</t>
+        </is>
+      </c>
+      <c r="H261" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22T14:42:23+00:00</t>
+        </is>
+      </c>
       <c r="I261" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/farion1231/cc-switch/releases</t>
+          <t>https://github.com/farion1231/cc-switch/releases/tag/v3.20.4</t>
         </is>
       </c>
       <c r="J261" s="2" t="inlineStr"/>
@@ -9747,13 +10187,17 @@
       </c>
       <c r="G262" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H262" s="3" t="inlineStr"/>
+          <t>v30.0</t>
+        </is>
+      </c>
+      <c r="H262" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-13T12:46:30+00:00</t>
+        </is>
+      </c>
       <c r="I262" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bitcoin/bitcoin/releases</t>
+          <t>https://github.com/bitcoin/bitcoin/releases/tag/v30.0</t>
         </is>
       </c>
       <c r="J262" s="2" t="inlineStr"/>
@@ -9780,13 +10224,17 @@
       </c>
       <c r="G263" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H263" s="3" t="inlineStr"/>
+          <t>v30.1</t>
+        </is>
+      </c>
+      <c r="H263" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-02T16:15:41+00:00</t>
+        </is>
+      </c>
       <c r="I263" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bitcoin/bitcoin/releases</t>
+          <t>https://github.com/bitcoin/bitcoin/releases/tag/v30.1</t>
         </is>
       </c>
       <c r="J263" s="2" t="inlineStr"/>
@@ -9813,13 +10261,17 @@
       </c>
       <c r="G264" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H264" s="3" t="inlineStr"/>
+          <t>v29.3</t>
+        </is>
+      </c>
+      <c r="H264" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-11T11:04:13+00:00</t>
+        </is>
+      </c>
       <c r="I264" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bitcoin/bitcoin/releases</t>
+          <t>https://github.com/bitcoin/bitcoin/releases/tag/v29.3</t>
         </is>
       </c>
       <c r="J264" s="2" t="inlineStr"/>
@@ -9846,13 +10298,17 @@
       </c>
       <c r="G265" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H265" s="3" t="inlineStr"/>
+          <t>v31.1</t>
+        </is>
+      </c>
+      <c r="H265" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08T09:14:15+00:00</t>
+        </is>
+      </c>
       <c r="I265" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bitcoin/bitcoin/releases</t>
+          <t>https://github.com/bitcoin/bitcoin/releases/tag/v31.1</t>
         </is>
       </c>
       <c r="J265" s="2" t="inlineStr"/>
@@ -9879,13 +10335,17 @@
       </c>
       <c r="G266" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H266" s="3" t="inlineStr"/>
+          <t>v30.3</t>
+        </is>
+      </c>
+      <c r="H266" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10T09:34:59+00:00</t>
+        </is>
+      </c>
       <c r="I266" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/bitcoin/bitcoin/releases</t>
+          <t>https://github.com/bitcoin/bitcoin/releases/tag/v30.3</t>
         </is>
       </c>
       <c r="J266" s="2" t="inlineStr"/>
@@ -9912,13 +10372,17 @@
       </c>
       <c r="G267" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H267" s="3" t="inlineStr"/>
+          <t>v0.6.6</t>
+        </is>
+      </c>
+      <c r="H267" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:19:01+00:00</t>
+        </is>
+      </c>
       <c r="I267" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/heygen-com/hyperframes/releases</t>
+          <t>https://github.com/heygen-com/hyperframes/releases/tag/v0.6.6</t>
         </is>
       </c>
       <c r="J267" s="2" t="inlineStr"/>
@@ -9945,13 +10409,17 @@
       </c>
       <c r="G268" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H268" s="3" t="inlineStr"/>
+          <t>v0.6.74</t>
+        </is>
+      </c>
+      <c r="H268" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-05T22:44:01+00:00</t>
+        </is>
+      </c>
       <c r="I268" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/heygen-com/hyperframes/releases</t>
+          <t>https://github.com/heygen-com/hyperframes/releases/tag/v0.6.74</t>
         </is>
       </c>
       <c r="J268" s="2" t="inlineStr"/>
@@ -9978,13 +10446,17 @@
       </c>
       <c r="G269" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H269" s="3" t="inlineStr"/>
+          <t>v0.6.96</t>
+        </is>
+      </c>
+      <c r="H269" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-13T03:32:25+00:00</t>
+        </is>
+      </c>
       <c r="I269" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/heygen-com/hyperframes/releases</t>
+          <t>https://github.com/heygen-com/hyperframes/releases/tag/v0.6.96</t>
         </is>
       </c>
       <c r="J269" s="2" t="inlineStr"/>
@@ -10011,13 +10483,17 @@
       </c>
       <c r="G270" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H270" s="3" t="inlineStr"/>
+          <t>v0.7.38</t>
+        </is>
+      </c>
+      <c r="H270" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07T00:52:19+00:00</t>
+        </is>
+      </c>
       <c r="I270" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/heygen-com/hyperframes/releases</t>
+          <t>https://github.com/heygen-com/hyperframes/releases/tag/v0.7.38</t>
         </is>
       </c>
       <c r="J270" s="2" t="inlineStr"/>
@@ -10044,13 +10520,17 @@
       </c>
       <c r="G271" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H271" s="3" t="inlineStr"/>
+          <t>v0.8.53</t>
+        </is>
+      </c>
+      <c r="H271" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-20T03:34:41+00:00</t>
+        </is>
+      </c>
       <c r="I271" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/heygen-com/hyperframes/releases</t>
+          <t>https://github.com/heygen-com/hyperframes/releases/tag/v0.8.53</t>
         </is>
       </c>
       <c r="J271" s="2" t="inlineStr"/>
@@ -10077,13 +10557,17 @@
       </c>
       <c r="G272" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H272" s="3" t="inlineStr"/>
+          <t>n8n@2.7.3</t>
+        </is>
+      </c>
+      <c r="H272" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-09T08:18:12+00:00</t>
+        </is>
+      </c>
       <c r="I272" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/n8n-io/n8n/releases</t>
+          <t>https://github.com/n8n-io/n8n/releases/tag/n8n@2.7.3</t>
         </is>
       </c>
       <c r="J272" s="2" t="inlineStr"/>
@@ -10110,13 +10594,17 @@
       </c>
       <c r="G273" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H273" s="3" t="inlineStr"/>
+          <t>n8n@1.123.42</t>
+        </is>
+      </c>
+      <c r="H273" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08T09:21:48+00:00</t>
+        </is>
+      </c>
       <c r="I273" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/n8n-io/n8n/releases</t>
+          <t>https://github.com/n8n-io/n8n/releases/tag/n8n@1.123.42</t>
         </is>
       </c>
       <c r="J273" s="2" t="inlineStr"/>
@@ -10143,13 +10631,17 @@
       </c>
       <c r="G274" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H274" s="3" t="inlineStr"/>
+          <t>n8n@1.123.59</t>
+        </is>
+      </c>
+      <c r="H274" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-19T10:31:00+00:00</t>
+        </is>
+      </c>
       <c r="I274" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/n8n-io/n8n/releases</t>
+          <t>https://github.com/n8n-io/n8n/releases/tag/n8n@1.123.59</t>
         </is>
       </c>
       <c r="J274" s="2" t="inlineStr"/>
@@ -10176,13 +10668,17 @@
       </c>
       <c r="G275" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H275" s="3" t="inlineStr"/>
+          <t>n8n@2.28.3</t>
+        </is>
+      </c>
+      <c r="H275" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29T08:14:13+00:00</t>
+        </is>
+      </c>
       <c r="I275" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/n8n-io/n8n/releases</t>
+          <t>https://github.com/n8n-io/n8n/releases/tag/n8n@2.28.3</t>
         </is>
       </c>
       <c r="J275" s="2" t="inlineStr"/>
@@ -10209,13 +10705,17 @@
       </c>
       <c r="G276" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H276" s="3" t="inlineStr"/>
+          <t>n8n@1.123.76</t>
+        </is>
+      </c>
+      <c r="H276" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02T07:37:28+00:00</t>
+        </is>
+      </c>
       <c r="I276" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/n8n-io/n8n/releases</t>
+          <t>https://github.com/n8n-io/n8n/releases/tag/n8n@1.123.76</t>
         </is>
       </c>
       <c r="J276" s="2" t="inlineStr"/>
@@ -10242,13 +10742,17 @@
       </c>
       <c r="G277" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H277" s="3" t="inlineStr"/>
+          <t>svelte@5.41.1</t>
+        </is>
+      </c>
+      <c r="H277" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-20T13:32:28+00:00</t>
+        </is>
+      </c>
       <c r="I277" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/sveltejs/svelte/releases</t>
+          <t>https://github.com/sveltejs/svelte/releases/tag/svelte@5.41.1</t>
         </is>
       </c>
       <c r="J277" s="2" t="inlineStr"/>
@@ -10275,13 +10779,17 @@
       </c>
       <c r="G278" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H278" s="3" t="inlineStr"/>
+          <t>svelte@5.41.3</t>
+        </is>
+      </c>
+      <c r="H278" s="3" t="inlineStr">
+        <is>
+          <t>2025-10-23T18:51:00+00:00</t>
+        </is>
+      </c>
       <c r="I278" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/sveltejs/svelte/releases</t>
+          <t>https://github.com/sveltejs/svelte/releases/tag/svelte@5.41.3</t>
         </is>
       </c>
       <c r="J278" s="2" t="inlineStr"/>
@@ -10308,13 +10816,17 @@
       </c>
       <c r="G279" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H279" s="3" t="inlineStr"/>
+          <t>svelte@5.48.0</t>
+        </is>
+      </c>
+      <c r="H279" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-22T03:05:13+00:00</t>
+        </is>
+      </c>
       <c r="I279" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/sveltejs/svelte/releases</t>
+          <t>https://github.com/sveltejs/svelte/releases/tag/svelte@5.48.0</t>
         </is>
       </c>
       <c r="J279" s="2" t="inlineStr"/>
@@ -10341,13 +10853,17 @@
       </c>
       <c r="G280" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H280" s="3" t="inlineStr"/>
+          <t>svelte@5.51.4</t>
+        </is>
+      </c>
+      <c r="H280" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-18T17:52:24+00:00</t>
+        </is>
+      </c>
       <c r="I280" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/sveltejs/svelte/releases</t>
+          <t>https://github.com/sveltejs/svelte/releases/tag/svelte@5.51.4</t>
         </is>
       </c>
       <c r="J280" s="2" t="inlineStr"/>
@@ -10374,13 +10890,17 @@
       </c>
       <c r="G281" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H281" s="3" t="inlineStr"/>
+          <t>svelte@5.55.2</t>
+        </is>
+      </c>
+      <c r="H281" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-07T19:53:53+00:00</t>
+        </is>
+      </c>
       <c r="I281" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/sveltejs/svelte/releases</t>
+          <t>https://github.com/sveltejs/svelte/releases/tag/svelte@5.55.2</t>
         </is>
       </c>
       <c r="J281" s="2" t="inlineStr"/>
@@ -10407,13 +10927,17 @@
       </c>
       <c r="G282" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H282" s="3" t="inlineStr"/>
+          <t>@upstash/context7-mcp@2.1.1</t>
+        </is>
+      </c>
+      <c r="H282" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-29T08:49:41+00:00</t>
+        </is>
+      </c>
       <c r="I282" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/upstash/context7/releases</t>
+          <t>https://github.com/upstash/context7/releases/tag/@upstash/context7-mcp@2.1.1</t>
         </is>
       </c>
       <c r="J282" s="2" t="inlineStr"/>
@@ -10440,13 +10964,17 @@
       </c>
       <c r="G283" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H283" s="3" t="inlineStr"/>
+          <t>ctx7@0.3.1</t>
+        </is>
+      </c>
+      <c r="H283" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-18T13:34:48+00:00</t>
+        </is>
+      </c>
       <c r="I283" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/upstash/context7/releases</t>
+          <t>https://github.com/upstash/context7/releases/tag/ctx7@0.3.1</t>
         </is>
       </c>
       <c r="J283" s="2" t="inlineStr"/>
@@ -10473,13 +11001,17 @@
       </c>
       <c r="G284" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H284" s="3" t="inlineStr"/>
+          <t>ctx7@0.3.8</t>
+        </is>
+      </c>
+      <c r="H284" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-27T14:17:41+00:00</t>
+        </is>
+      </c>
       <c r="I284" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/upstash/context7/releases</t>
+          <t>https://github.com/upstash/context7/releases/tag/ctx7@0.3.8</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr"/>
@@ -10506,13 +11038,17 @@
       </c>
       <c r="G285" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H285" s="3" t="inlineStr"/>
+          <t>ctx7@0.4.3</t>
+        </is>
+      </c>
+      <c r="H285" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21T09:46:24+00:00</t>
+        </is>
+      </c>
       <c r="I285" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/upstash/context7/releases</t>
+          <t>https://github.com/upstash/context7/releases/tag/ctx7@0.4.3</t>
         </is>
       </c>
       <c r="J285" s="2" t="inlineStr"/>
@@ -10539,13 +11075,17 @@
       </c>
       <c r="G286" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H286" s="3" t="inlineStr"/>
+          <t>ctx7@0.5.9</t>
+        </is>
+      </c>
+      <c r="H286" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-27T08:21:42+00:00</t>
+        </is>
+      </c>
       <c r="I286" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/upstash/context7/releases</t>
+          <t>https://github.com/upstash/context7/releases/tag/ctx7@0.5.9</t>
         </is>
       </c>
       <c r="J286" s="2" t="inlineStr"/>
@@ -10572,13 +11112,17 @@
       </c>
       <c r="G287" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H287" s="3" t="inlineStr"/>
+          <t>v0.2.0</t>
+        </is>
+      </c>
+      <c r="H287" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-19T15:55:08+00:00</t>
+        </is>
+      </c>
       <c r="I287" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/THU-MAIC/OpenMAIC/releases</t>
+          <t>https://github.com/THU-MAIC/OpenMAIC/releases/tag/v0.2.0</t>
         </is>
       </c>
       <c r="J287" s="2" t="inlineStr"/>
@@ -10605,13 +11149,17 @@
       </c>
       <c r="G288" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H288" s="3" t="inlineStr"/>
+          <t>v0.2.1</t>
+        </is>
+      </c>
+      <c r="H288" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-26T16:12:06+00:00</t>
+        </is>
+      </c>
       <c r="I288" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/THU-MAIC/OpenMAIC/releases</t>
+          <t>https://github.com/THU-MAIC/OpenMAIC/releases/tag/v0.2.1</t>
         </is>
       </c>
       <c r="J288" s="2" t="inlineStr"/>
@@ -10638,13 +11186,17 @@
       </c>
       <c r="G289" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H289" s="3" t="inlineStr"/>
+          <t>v1.1.0</t>
+        </is>
+      </c>
+      <c r="H289" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24T06:04:48+00:00</t>
+        </is>
+      </c>
       <c r="I289" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/THU-MAIC/OpenMAIC/releases</t>
+          <t>https://github.com/THU-MAIC/OpenMAIC/releases/tag/v1.1.0</t>
         </is>
       </c>
       <c r="J289" s="2" t="inlineStr"/>
@@ -10671,13 +11223,17 @@
       </c>
       <c r="G290" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H290" s="3" t="inlineStr"/>
+          <t>v1.1.1</t>
+        </is>
+      </c>
+      <c r="H290" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-26T16:20:13+00:00</t>
+        </is>
+      </c>
       <c r="I290" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/THU-MAIC/OpenMAIC/releases</t>
+          <t>https://github.com/THU-MAIC/OpenMAIC/releases/tag/v1.1.1</t>
         </is>
       </c>
       <c r="J290" s="2" t="inlineStr"/>
@@ -10704,13 +11260,17 @@
       </c>
       <c r="G291" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H291" s="3" t="inlineStr"/>
+          <t>v1.1.2</t>
+        </is>
+      </c>
+      <c r="H291" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-28T10:10:50+00:00</t>
+        </is>
+      </c>
       <c r="I291" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/THU-MAIC/OpenMAIC/releases</t>
+          <t>https://github.com/THU-MAIC/OpenMAIC/releases/tag/v1.1.2</t>
         </is>
       </c>
       <c r="J291" s="2" t="inlineStr"/>
@@ -10737,13 +11297,17 @@
       </c>
       <c r="G292" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H292" s="3" t="inlineStr"/>
+          <t>v0.3.12</t>
+        </is>
+      </c>
+      <c r="H292" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-04T00:53:14+00:00</t>
+        </is>
+      </c>
       <c r="I292" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/codewhale-hq/Codewhale/releases</t>
+          <t>https://github.com/codewhale-hq/Codewhale/releases/tag/v0.3.12</t>
         </is>
       </c>
       <c r="J292" s="2" t="inlineStr"/>
@@ -10770,13 +11334,17 @@
       </c>
       <c r="G293" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H293" s="3" t="inlineStr"/>
+          <t>v0.3.24</t>
+        </is>
+      </c>
+      <c r="H293" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-26T20:25:30+00:00</t>
+        </is>
+      </c>
       <c r="I293" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/codewhale-hq/Codewhale/releases</t>
+          <t>https://github.com/codewhale-hq/Codewhale/releases/tag/v0.3.24</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr"/>
@@ -10803,13 +11371,17 @@
       </c>
       <c r="G294" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H294" s="3" t="inlineStr"/>
+          <t>v0.4.5</t>
+        </is>
+      </c>
+      <c r="H294" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-24T16:59:25+00:00</t>
+        </is>
+      </c>
       <c r="I294" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/codewhale-hq/Codewhale/releases</t>
+          <t>https://github.com/codewhale-hq/Codewhale/releases/tag/v0.4.5</t>
         </is>
       </c>
       <c r="J294" s="2" t="inlineStr"/>
@@ -10836,13 +11408,17 @@
       </c>
       <c r="G295" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H295" s="3" t="inlineStr"/>
+          <t>v0.9.0</t>
+        </is>
+      </c>
+      <c r="H295" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16T20:05:39+00:00</t>
+        </is>
+      </c>
       <c r="I295" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/codewhale-hq/Codewhale/releases</t>
+          <t>https://github.com/codewhale-hq/Codewhale/releases/tag/v0.9.0</t>
         </is>
       </c>
       <c r="J295" s="2" t="inlineStr"/>
@@ -10869,13 +11445,17 @@
       </c>
       <c r="G296" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H296" s="3" t="inlineStr"/>
+          <t>v0.9.6</t>
+        </is>
+      </c>
+      <c r="H296" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-12T08:47:19+00:00</t>
+        </is>
+      </c>
       <c r="I296" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/codewhale-hq/Codewhale/releases</t>
+          <t>https://github.com/codewhale-hq/Codewhale/releases/tag/v0.9.6</t>
         </is>
       </c>
       <c r="J296" s="2" t="inlineStr"/>
@@ -10902,13 +11482,17 @@
       </c>
       <c r="G297" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H297" s="3" t="inlineStr"/>
+          <t>v1.33.1</t>
+        </is>
+      </c>
+      <c r="H297" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-20T14:24:56+00:00</t>
+        </is>
+      </c>
       <c r="I297" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/meilisearch/meilisearch/releases</t>
+          <t>https://github.com/meilisearch/meilisearch/releases/tag/v1.33.1</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr"/>
@@ -10935,13 +11519,17 @@
       </c>
       <c r="G298" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H298" s="3" t="inlineStr"/>
+          <t>v1.34.1</t>
+        </is>
+      </c>
+      <c r="H298" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-27T09:32:44+00:00</t>
+        </is>
+      </c>
       <c r="I298" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/meilisearch/meilisearch/releases</t>
+          <t>https://github.com/meilisearch/meilisearch/releases/tag/v1.34.1</t>
         </is>
       </c>
       <c r="J298" s="2" t="inlineStr"/>
@@ -10968,13 +11556,17 @@
       </c>
       <c r="G299" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H299" s="3" t="inlineStr"/>
+          <t>v1.34.2</t>
+        </is>
+      </c>
+      <c r="H299" s="3" t="inlineStr">
+        <is>
+          <t>2026-01-28T08:20:49+00:00</t>
+        </is>
+      </c>
       <c r="I299" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/meilisearch/meilisearch/releases</t>
+          <t>https://github.com/meilisearch/meilisearch/releases/tag/v1.34.2</t>
         </is>
       </c>
       <c r="J299" s="2" t="inlineStr"/>
@@ -11001,13 +11593,17 @@
       </c>
       <c r="G300" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H300" s="3" t="inlineStr"/>
+          <t>v1.35.0</t>
+        </is>
+      </c>
+      <c r="H300" s="3" t="inlineStr">
+        <is>
+          <t>2026-02-02T09:57:03+00:00</t>
+        </is>
+      </c>
       <c r="I300" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/meilisearch/meilisearch/releases</t>
+          <t>https://github.com/meilisearch/meilisearch/releases/tag/v1.35.0</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr"/>
@@ -11034,13 +11630,17 @@
       </c>
       <c r="G301" s="3" t="inlineStr">
         <is>
-          <t>(pendente de persistência)</t>
-        </is>
-      </c>
-      <c r="H301" s="3" t="inlineStr"/>
+          <t>v1.50.0</t>
+        </is>
+      </c>
+      <c r="H301" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20T08:54:18+00:00</t>
+        </is>
+      </c>
       <c r="I301" s="4" t="inlineStr">
         <is>
-          <t>https://github.com/meilisearch/meilisearch/releases</t>
+          <t>https://github.com/meilisearch/meilisearch/releases/tag/v1.50.0</t>
         </is>
       </c>
       <c r="J301" s="2" t="inlineStr"/>
@@ -11705,7 +12305,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>2026-10-15 20:47:29</t>
+          <t>2026-10-20 21:32:59</t>
         </is>
       </c>
     </row>

</xml_diff>